<commit_message>
Add universe H for financials and real estate, move Government to C2, exclude US outside E, restore project instruction, rewrite prompt 13
</commit_message>
<xml_diff>
--- a/05-Resources/Templates/02-Screening.xlsx
+++ b/05-Resources/Templates/02-Screening.xlsx
@@ -608,7 +608,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Begin met universum A, de hoofdroute. B tot en met F zijn vangnetten voor bedrijven die A bewust buiten laat, G is het aparte universum voor life sciences, en de drie landenlijsten zijn voor een kijkje buiten de hoofdroute.</t>
+          <t>Begin met universum A, de hoofdroute. D, E en F gebruiken dezelfde industrieën als A; B, C, G en H zijn de vangnetten voor de industrieën die A buiten laat. Alleen E kijkt naar de Verenigde Staten. De drie landenlijsten zijn voor een kijkje buiten de hoofdroute.</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Universums: de zeven universums en drie landenlijsten met hun instellingen als naslag bij het invullen</t>
+          <t>Universums: de acht universums en drie landenlijsten met hun instellingen als naslag bij het invullen</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1039,7 +1039,7 @@
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>Landenlijst Nederland</t>
+          <t>H. Financials en vastgoed</t>
         </is>
       </c>
       <c r="B21" s="10" t="n"/>
@@ -1054,7 +1054,7 @@
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>Landenlijst Hongkong</t>
+          <t>Landenlijst Nederland</t>
         </is>
       </c>
       <c r="B22" s="10" t="n"/>
@@ -1069,7 +1069,7 @@
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>Landenlijst Verenigde Staten</t>
+          <t>Landenlijst Hongkong</t>
         </is>
       </c>
       <c r="B23" s="10" t="n"/>
@@ -1081,173 +1081,188 @@
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>Landenlijst Verenigde Staten</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="n"/>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="10" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="16">
+        <f>COUNTIF(Kandidaten!$I$2:$I$121,A24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Uitkomst</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>Aantal namen ruw, alle lijsten samen</t>
-        </is>
-      </c>
-      <c r="B26" s="17">
-        <f>IF(SUM(E14:E23)=0,"",SUM(E14:E23))</f>
-        <v/>
-      </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
-          <t>Ongeveer honderd is doorgaans genoeg voor vijf tot tien kandidaten.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Aantal kandidaten ingevuld</t>
+          <t>Aantal namen ruw, alle lijsten samen</t>
         </is>
       </c>
       <c r="B27" s="17">
-        <f>COUNTA(Kandidaten!$B$2:$B$121)</f>
-        <v/>
+        <f>IF(SUM(E14:E24)=0,"",SUM(E14:E24))</f>
+        <v/>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Ongeveer honderd is doorgaans genoeg voor vijf tot tien kandidaten.</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Waarvan volgende stap Snelle analyse</t>
+          <t>Aantal kandidaten ingevuld</t>
         </is>
       </c>
       <c r="B28" s="17">
-        <f>COUNTIF(Kandidaten!$W$2:$W$121,"Snelle analyse")</f>
+        <f>COUNTA(Kandidaten!$B$2:$B$121)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Waarvan Later terugkomen</t>
+          <t>Waarvan volgende stap Snelle analyse</t>
         </is>
       </c>
       <c r="B29" s="17">
-        <f>COUNTIF(Kandidaten!$W$2:$W$121,"Later terugkomen")</f>
+        <f>COUNTIF(Kandidaten!$W$2:$W$121,"Snelle analyse")</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
+          <t>Waarvan Later terugkomen</t>
+        </is>
+      </c>
+      <c r="B30" s="17">
+        <f>COUNTIF(Kandidaten!$W$2:$W$121,"Later terugkomen")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
           <t>Waarvan Stoppen</t>
         </is>
       </c>
-      <c r="B30" s="17">
+      <c r="B31" s="17">
         <f>COUNTIF(Kandidaten!$W$2:$W$121,"Stoppen")</f>
         <v/>
       </c>
     </row>
-    <row r="31" ht="60" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+    <row r="32" ht="60" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>Uitzonderingen op de filters die ik heb toegelaten</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="n"/>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>Een naam die buiten een filter viel maar toch op de lijst staat, met de reden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>Conclusie van de ronde</t>
         </is>
       </c>
       <c r="B32" s="10" t="n"/>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Kies uit de lijst.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="60" customHeight="1">
+          <t>Een naam die buiten een filter viel maar toch op de lijst staat, met de reden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>Wat ik volgende ronde bewust anders doe</t>
+          <t>Conclusie van de ronde</t>
         </is>
       </c>
       <c r="B33" s="10" t="n"/>
       <c r="C33" s="11" t="inlineStr">
         <is>
+          <t>Kies uit de lijst.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="60" customHeight="1">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Wat ik volgende ronde bewust anders doe</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
           <t>Eén of enkele instellingen, met het verwachte effect.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Controles</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>Conclusie tegenover het aantal met Snelle analyse</t>
-        </is>
-      </c>
-      <c r="B36" s="18">
-        <f>IF(B32="","",IF(AND(B32="Vijf tot tien kandidaten",OR(B28&lt;5,B28&gt;10)),"Verschilt: controleer","Komt overeen"))</f>
-        <v/>
-      </c>
-      <c r="C36" s="11" t="inlineStr">
-        <is>
-          <t>Vijf tot tien is een richtlijn; een afwijking vraagt een reden, geen correctie van de conclusie.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>Kandidaten zonder reden om verder te kijken</t>
-        </is>
-      </c>
-      <c r="B37" s="19">
-        <f>COUNTIFS(Kandidaten!$B$2:$B$121,"&lt;&gt;",Kandidaten!$V$2:$V$121,"")</f>
+          <t>Conclusie tegenover het aantal met Snelle analyse</t>
+        </is>
+      </c>
+      <c r="B37" s="18">
+        <f>IF(B33="","",IF(AND(B33="Vijf tot tien kandidaten",OR(B29&lt;5,B29&gt;10)),"Verschilt: controleer","Komt overeen"))</f>
         <v/>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Een naam zonder reden hoort niet op de lijst.</t>
+          <t>Vijf tot tien is een richtlijn; een afwijking vraagt een reden, geen correctie van de conclusie.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>Kandidaten zonder universum of landenlijst</t>
+          <t>Kandidaten zonder reden om verder te kijken</t>
         </is>
       </c>
       <c r="B38" s="19">
-        <f>COUNTIFS(Kandidaten!$B$2:$B$121,"&lt;&gt;",Kandidaten!$I$2:$I$121,"")</f>
-        <v/>
+        <f>COUNTIFS(Kandidaten!$B$2:$B$121,"&lt;&gt;",Kandidaten!$V$2:$V$121,"")</f>
+        <v/>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Een naam zonder reden hoort niet op de lijst.</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
+          <t>Kandidaten zonder universum of landenlijst</t>
+        </is>
+      </c>
+      <c r="B39" s="19">
+        <f>COUNTIFS(Kandidaten!$B$2:$B$121,"&lt;&gt;",Kandidaten!$I$2:$I$121,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
           <t>Kandidaten zonder controle op verhandelbaarheid</t>
         </is>
       </c>
-      <c r="B39" s="19">
+      <c r="B40" s="19">
         <f>COUNTIFS(Kandidaten!$B$2:$B$121,"&lt;&gt;",Kandidaten!$N$2:$N$121,"")</f>
         <v/>
       </c>
-      <c r="C39" s="11" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>Check 1 hoort bij het screenen, niet bij de snelle analyse.</t>
         </is>
@@ -1255,10 +1270,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B14:B23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige waarde" error="Kies een waarde uit de lijst." type="list">
+    <dataValidation sqref="B14:B24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige waarde" error="Kies een waarde uit de lijst." type="list">
       <formula1>"Ja,Nee"</formula1>
     </dataValidation>
-    <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige waarde" error="Kies een waarde uit de lijst." type="list">
+    <dataValidation sqref="B33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige waarde" error="Kies een waarde uit de lijst." type="list">
       <formula1>"Vijf tot tien kandidaten,Geen geschikte selectie nu"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5159,7 +5174,7 @@
   <autoFilter ref="A1:Z121"/>
   <dataValidations count="4">
     <dataValidation sqref="I2:I121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige waarde" error="Kies een waarde uit de lijst." type="list">
-      <formula1>"A. Snelle groeiers,B. Cyclische bedrijven,C. Gereguleerde bedrijven,D. Omzetgroei zonder winst,E. Amerikaanse smallcaps,F. Midcaps,G. Life Sciences,Landenlijst Nederland,Landenlijst Hongkong,Landenlijst Verenigde Staten"</formula1>
+      <formula1>"A. Snelle groeiers,B. Cyclische bedrijven,C. Gereguleerde bedrijven,D. Omzetgroei zonder winst,E. Amerikaanse smallcaps,F. Midcaps,G. Life Sciences,H. Financials en vastgoed,Landenlijst Nederland,Landenlijst Hongkong,Landenlijst Verenigde Staten"</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige waarde" error="Kies een waarde uit de lijst." type="list">
       <formula1>"Ja,Nee,Onbekend"</formula1>
@@ -9806,7 +9821,7 @@
   <autoFilter ref="A1:AC121"/>
   <dataValidations count="5">
     <dataValidation sqref="D2:D121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige waarde" error="Kies een waarde uit de lijst." type="list">
-      <formula1>"A. Snelle groeiers,B. Cyclische bedrijven,C. Gereguleerde bedrijven,D. Omzetgroei zonder winst,E. Amerikaanse smallcaps,F. Midcaps,G. Life Sciences,Landenlijst Nederland,Landenlijst Hongkong,Landenlijst Verenigde Staten"</formula1>
+      <formula1>"A. Snelle groeiers,B. Cyclische bedrijven,C. Gereguleerde bedrijven,D. Omzetgroei zonder winst,E. Amerikaanse smallcaps,F. Midcaps,G. Life Sciences,H. Financials en vastgoed,Landenlijst Nederland,Landenlijst Hongkong,Landenlijst Verenigde Staten"</formula1>
     </dataValidation>
     <dataValidation sqref="X2:X121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ongeldige waarde" error="Kies een waarde uit de lijst." type="list">
       <formula1>"Ja,Nee"</formula1>
@@ -9831,7 +9846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -9908,7 +9923,7 @@
       </c>
       <c r="C3" s="28" t="inlineStr">
         <is>
-          <t>Alle DeGiro-landen, inclusief de Verenigde Staten</t>
+          <t>Alle DeGiro-landen behalve de Verenigde Staten</t>
         </is>
       </c>
       <c r="D3" s="28" t="inlineStr">
@@ -9935,7 +9950,7 @@
       </c>
       <c r="C4" s="28" t="inlineStr">
         <is>
-          <t>Alle DeGiro-landen, inclusief de Verenigde Staten</t>
+          <t>Alle DeGiro-landen behalve de Verenigde Staten</t>
         </is>
       </c>
       <c r="D4" s="28" t="inlineStr">
@@ -9945,7 +9960,7 @@
       </c>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>C1: Utilities alle industrieën, Communications alle industrieën, Transportation: Railroads, Airlines, Other Transportation, Industrial Services: Oil &amp; Gas Pipelines, Environmental Services. C2: Electronic Technology: Aerospace &amp; Defense, Health Services: Hospital/Nursing Management, Managed Health Care, Medical/Nursing Services, Consumer Services: Casinos/Gaming, Consumer Non-Durables: Tobacco</t>
+          <t>C1: Utilities alle industrieën, Communications alle industrieën, Transportation: Railroads, Airlines, Other Transportation, Industrial Services: Oil &amp; Gas Pipelines, Environmental Services. C2: Electronic Technology: Aerospace &amp; Defense, Health Services: Hospital/Nursing Management, Managed Health Care, Medical/Nursing Services, Consumer Services: Casinos/Gaming, Consumer Non-Durables: Tobacco, Government: Sovereign</t>
         </is>
       </c>
     </row>
@@ -9962,7 +9977,7 @@
       </c>
       <c r="C5" s="28" t="inlineStr">
         <is>
-          <t>Alle DeGiro-landen in Europa en Noord-Amerika, inclusief de Verenigde Staten</t>
+          <t>De DeGiro-landen in Europa, en Canada; niet de Verenigde Staten</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
@@ -9999,7 +10014,7 @@
       </c>
       <c r="E6" s="28" t="inlineStr">
         <is>
-          <t>Als bij A: de sectoren van B, C en G staan standaard uit</t>
+          <t>Als bij A, D en F</t>
         </is>
       </c>
     </row>
@@ -10038,12 +10053,12 @@
       </c>
       <c r="B8" s="28" t="inlineStr">
         <is>
-          <t>Apart universum: farmacie, biotechnologie en medische technologie, met koersen die op een goedkeuring of studie-uitkomst kunnen omslaan</t>
+          <t>Vangnet: farmacie, biotechnologie en medische technologie, met koersen die op een goedkeuring of studie-uitkomst kunnen omslaan</t>
         </is>
       </c>
       <c r="C8" s="28" t="inlineStr">
         <is>
-          <t>Alle DeGiro-landen, inclusief de Verenigde Staten</t>
+          <t>Alle DeGiro-landen behalve de Verenigde Staten</t>
         </is>
       </c>
       <c r="D8" s="28" t="inlineStr">
@@ -10060,34 +10075,34 @@
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
         <is>
-          <t>Landenlijst Nederland</t>
+          <t>H. Financials en vastgoed</t>
         </is>
       </c>
       <c r="B9" s="28" t="inlineStr">
         <is>
-          <t>Buiten de hoofdroute: persoonlijke interesse en eigen informatiebronnen</t>
+          <t>Vangnet: banken, verzekeraars, vastgoed, financiële dienstverleners en fondsen, met een eigen manier van waarderen</t>
         </is>
       </c>
       <c r="C9" s="28" t="inlineStr">
         <is>
-          <t>Nederland: Euronext Amsterdam</t>
+          <t>Alle DeGiro-landen behalve de Verenigde Staten</t>
         </is>
       </c>
       <c r="D9" s="28" t="inlineStr">
         <is>
-          <t>Geen ondergrens voor Market capitalization; geen groeifilters</t>
+          <t>H1 banken en verzekeraars: Market capitalization 500 miljoen tot 30 miljard dollar; Price to book ratio 0 tot 1,5; Return on equity % meer dan 10; Price to earnings ratio 0 tot 12. H2 vastgoed: Market capitalization 300 miljoen tot 10 miljard dollar; Price to book ratio 0 tot 1,2; Dividend yield % meer dan 4; Debt to equity ratio onder 1,5. H3 dienstverleners en fondsen: Market capitalization 300 miljoen tot 10 miljard dollar; Revenue growth % meer dan 8; Net margin % meer dan 10; Return on equity % meer dan 12; Price to earnings ratio 0 tot 25; Debt to equity ratio onder 1</t>
         </is>
       </c>
       <c r="E9" s="28" t="inlineStr">
         <is>
-          <t>Alle industrieën behalve Investment Trusts/Mutual Funds en Miscellaneous uit Miscellaneous, en Sovereign uit Government</t>
+          <t>H1: Finance: Major Banks, Regional Banks, Savings Banks, Property/Casualty Insurance, Multi-Line Insurance, Life/Health Insurance, Specialty Insurance. H2: Finance: Real Estate Investment Trusts, Real Estate Development. H3: Finance: Investment Managers, Investment Banks/Brokers, Insurance Brokers/Services, Financial Conglomerates, Finance/Rental/Leasing; Miscellaneous: Investment Trusts/Mutual Funds, Miscellaneous</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
         <is>
-          <t>Landenlijst Hongkong</t>
+          <t>Landenlijst Nederland</t>
         </is>
       </c>
       <c r="B10" s="28" t="inlineStr">
@@ -10097,57 +10112,84 @@
       </c>
       <c r="C10" s="28" t="inlineStr">
         <is>
-          <t>Hongkong: Hong Kong Stock Exchange</t>
+          <t>Nederland: Euronext Amsterdam</t>
         </is>
       </c>
       <c r="D10" s="28" t="inlineStr">
         <is>
-          <t>Market capitalization meer dan 1 miljard dollar; Price × average volume boven 1 miljoen dollar; geen groeifilters</t>
+          <t>Geen ondergrens voor Market capitalization; geen groeifilters</t>
         </is>
       </c>
       <c r="E10" s="28" t="inlineStr">
         <is>
-          <t>Alle industrieën behalve Investment Trusts/Mutual Funds en Miscellaneous uit Miscellaneous, en Sovereign uit Government</t>
+          <t>Alle industrieën behalve Investment Trusts/Mutual Funds en Miscellaneous uit Miscellaneous</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
         <is>
+          <t>Landenlijst Hongkong</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>Buiten de hoofdroute: persoonlijke interesse en eigen informatiebronnen</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="inlineStr">
+        <is>
+          <t>Hongkong: Hong Kong Stock Exchange</t>
+        </is>
+      </c>
+      <c r="D11" s="28" t="inlineStr">
+        <is>
+          <t>Market capitalization meer dan 1 miljard dollar; Price × average volume boven 1 miljoen dollar; geen groeifilters</t>
+        </is>
+      </c>
+      <c r="E11" s="28" t="inlineStr">
+        <is>
+          <t>Alle industrieën behalve Investment Trusts/Mutual Funds en Miscellaneous uit Miscellaneous</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
           <t>Landenlijst Verenigde Staten</t>
         </is>
       </c>
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>Buiten de hoofdroute: persoonlijke interesse en eigen informatiebronnen</t>
         </is>
       </c>
-      <c r="C11" s="28" t="inlineStr">
+      <c r="C12" s="28" t="inlineStr">
         <is>
           <t>Verenigde Staten: NASDAQ, NYSE, NYSE American</t>
         </is>
       </c>
-      <c r="D11" s="28" t="inlineStr">
+      <c r="D12" s="28" t="inlineStr">
         <is>
           <t>Market capitalization meer dan 2 miljard dollar; kleinere bedrijven komen via D en E; geen groeifilters</t>
         </is>
       </c>
-      <c r="E11" s="28" t="inlineStr">
-        <is>
-          <t>Alle industrieën behalve Investment Trusts/Mutual Funds en Miscellaneous uit Miscellaneous, en Sovereign uit Government</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Altijd uit in de universums: alle 14 industrieën van Finance en de 2 van Miscellaneous, en Sovereign uit Government. In de landenlijsten blijft Finance aan ter informatie; Miscellaneous en Government staan ook daar uit. De sectortabel, de vinklijst per universum en de kolommen op het scherm staan in 05-Resources/Screeners/screeners.md.</t>
+      <c r="E12" s="28" t="inlineStr">
+        <is>
+          <t>Alle industrieën behalve Investment Trusts/Mutual Funds en Miscellaneous uit Miscellaneous</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>A, D, E en F delen dezelfde industrieën; B, C, G en H zijn de vangnetten voor de rest, en elke industrie hoort bij precies één van A, B, C, G en H. Alleen E bevat de Verenigde Staten. In de landenlijsten staat alleen Miscellaneous uit. De sectortabel, de vinklijst per universum en de kolommen op het scherm staan in 05-Resources/Screeners/screeners.md.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update universe A screener filters: 5-year revenue CAGR, net income growth, FY net margin, mandatory ROE, liquidity filter
</commit_message>
<xml_diff>
--- a/05-Resources/Templates/02-Screening.xlsx
+++ b/05-Resources/Templates/02-Screening.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding Projects\belegger-kees-methode\05-Resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D378FCBB-CBA9-409D-A2B8-238BBE29A229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4301044E-4D02-4C21-9B30-48ED1BBB85AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -208,9 +208,6 @@
     <t>Alle DeGiro-landen behalve de Verenigde Staten</t>
   </si>
   <si>
-    <t>Market capitalization 200 miljoen tot 5 miljard dollar; Revenue growth % (TTM, YoY) meer dan 12; Earnings per share diluted growth % (TTM, YoY) meer dan 18; Net margin % meer dan 5; Price to earnings ratio 0 tot 35; Return on equity % meer dan 12 (weglaten als de lijst te klein wordt)</t>
-  </si>
-  <si>
     <t>Market capitalization 200 miljoen tot 10 miljard dollar; Enterprise value to EBITDA ratio 0 tot 7; Debt to equity ratio onder 1; Free cash flow margin % boven 0; Current ratio boven 1. Niet op Price to earnings ratio filteren</t>
   </si>
   <si>
@@ -446,6 +443,9 @@
   </si>
   <si>
     <t>Status: werkversie, in gebruik bij de screeningronde van september 2026. Bijgewerkt op 15 september 2026. Auteur: Kees van Wanrooij, Belegger Kees.</t>
+  </si>
+  <si>
+    <t>Market capitalization 200 miljoen tot 5 miljard dollar; Price x average volume 10 dagen meer dan 50.000; Revenue growth 5 year CAGR meer dan 10; Net income growth % (TTM, YoY) meer dan 10; Net margin % (FY) meer dan 10; Return on equity % (TTM) meer dan 10; Price to earnings ratio onder 35</t>
   </si>
 </sst>
 </file>
@@ -631,7 +631,7 @@
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -698,6 +698,36 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -709,40 +739,6 @@
     </xf>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1460,7 +1456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A60"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="118" customWidth="1"/>
@@ -1471,9 +1467,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="35"/>
-    </row>
     <row r="3" spans="1:1">
       <c r="A3" s="23" t="s">
         <v>1</v>
@@ -1481,11 +1474,11 @@
     </row>
     <row r="4" spans="1:1" ht="25.5">
       <c r="A4" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" s="36"/>
+      <c r="A5" s="27"/>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="23" t="s">
@@ -1494,52 +1487,52 @@
     </row>
     <row r="7" spans="1:1" ht="25.5">
       <c r="A7" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="25.5">
       <c r="A9" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="38.25">
       <c r="A10" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="25.5">
       <c r="A11" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="38.25">
       <c r="A12" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="25.5">
       <c r="A13" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="26.25">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="28" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="26.25">
+      <c r="A15" s="29" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="26.25">
-      <c r="A15" s="38" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:1">
@@ -1551,28 +1544,28 @@
       <c r="A18" s="2"/>
     </row>
     <row r="19" spans="1:1">
-      <c r="A19" s="39" t="s">
+      <c r="A19" s="30" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" s="28" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="22" spans="1:1">
-      <c r="A22" s="37" t="s">
-        <v>111</v>
-      </c>
-    </row>
     <row r="23" spans="1:1">
-      <c r="A23" s="38" t="s">
-        <v>90</v>
+      <c r="A23" s="29" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="24" spans="1:1">
@@ -1580,7 +1573,7 @@
     </row>
     <row r="25" spans="1:1" ht="26.25">
       <c r="A25" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="26" spans="1:1">
@@ -1588,115 +1581,25 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:1">
-      <c r="A27" s="35"/>
-    </row>
     <row r="28" spans="1:1">
-      <c r="A28" s="39" t="s">
+      <c r="A28" s="30" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:1">
-      <c r="A29" s="37" t="s">
+      <c r="A29" s="28" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="30" spans="1:1">
-      <c r="A30" s="37" t="s">
+      <c r="A30" s="28" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:1">
-      <c r="A31" s="37" t="s">
+      <c r="A31" s="28" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="32" spans="1:1">
-      <c r="A32" s="35"/>
-    </row>
-    <row r="33" spans="1:1">
-      <c r="A33" s="35"/>
-    </row>
-    <row r="34" spans="1:1">
-      <c r="A34" s="35"/>
-    </row>
-    <row r="35" spans="1:1">
-      <c r="A35" s="35"/>
-    </row>
-    <row r="36" spans="1:1">
-      <c r="A36" s="35"/>
-    </row>
-    <row r="37" spans="1:1">
-      <c r="A37" s="35"/>
-    </row>
-    <row r="38" spans="1:1">
-      <c r="A38" s="35"/>
-    </row>
-    <row r="39" spans="1:1">
-      <c r="A39" s="35"/>
-    </row>
-    <row r="40" spans="1:1">
-      <c r="A40" s="35"/>
-    </row>
-    <row r="41" spans="1:1">
-      <c r="A41" s="35"/>
-    </row>
-    <row r="42" spans="1:1">
-      <c r="A42" s="35"/>
-    </row>
-    <row r="43" spans="1:1">
-      <c r="A43" s="35"/>
-    </row>
-    <row r="44" spans="1:1">
-      <c r="A44" s="35"/>
-    </row>
-    <row r="45" spans="1:1">
-      <c r="A45" s="35"/>
-    </row>
-    <row r="46" spans="1:1">
-      <c r="A46" s="35"/>
-    </row>
-    <row r="47" spans="1:1">
-      <c r="A47" s="35"/>
-    </row>
-    <row r="48" spans="1:1">
-      <c r="A48" s="35"/>
-    </row>
-    <row r="49" spans="1:1">
-      <c r="A49" s="35"/>
-    </row>
-    <row r="50" spans="1:1">
-      <c r="A50" s="35"/>
-    </row>
-    <row r="51" spans="1:1">
-      <c r="A51" s="35"/>
-    </row>
-    <row r="52" spans="1:1">
-      <c r="A52" s="35"/>
-    </row>
-    <row r="53" spans="1:1">
-      <c r="A53" s="35"/>
-    </row>
-    <row r="54" spans="1:1">
-      <c r="A54" s="35"/>
-    </row>
-    <row r="55" spans="1:1">
-      <c r="A55" s="35"/>
-    </row>
-    <row r="56" spans="1:1">
-      <c r="A56" s="35"/>
-    </row>
-    <row r="57" spans="1:1">
-      <c r="A57" s="35"/>
-    </row>
-    <row r="58" spans="1:1">
-      <c r="A58" s="35"/>
-    </row>
-    <row r="59" spans="1:1">
-      <c r="A59" s="35"/>
-    </row>
-    <row r="60" spans="1:1">
-      <c r="A60" s="35"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1730,22 +1633,22 @@
   <sheetData>
     <row r="1" spans="1:17" s="8" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A1" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>22</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>24</v>
@@ -1754,31 +1657,31 @@
         <v>25</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J1" s="6" t="s">
         <v>23</v>
       </c>
       <c r="K1" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="L1" s="6" t="s">
-        <v>65</v>
-      </c>
       <c r="M1" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O1" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P1" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:17">
@@ -1826,7 +1729,7 @@
         <f>IF(K3="","",IFERROR(VLOOKUP(J3,Fiat!$B$1:$C$20,2,FALSE)*K3,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
-      <c r="M3" s="32" t="str" cm="1">
+      <c r="M3" s="17" t="str" cm="1">
         <f t="array" ref="M3">IFERROR((_FV(C3,"Price")-_FV(C3,"52 week low",TRUE))/(_FV(C3,"52 week high",TRUE)-_FV(C3,"52 week low",TRUE)),"")</f>
         <v/>
       </c>
@@ -1855,7 +1758,7 @@
         <f>IF(K4="","",IFERROR(VLOOKUP(J4,Fiat!$B$1:$C$20,2,FALSE)*K4,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
-      <c r="M4" s="32" t="str" cm="1">
+      <c r="M4" s="17" t="str" cm="1">
         <f t="array" ref="M4">IFERROR((_FV(C4,"Price")-_FV(C4,"52 week low",TRUE))/(_FV(C4,"52 week high",TRUE)-_FV(C4,"52 week low",TRUE)),"")</f>
         <v/>
       </c>
@@ -1882,7 +1785,7 @@
         <f>IF(K5="","",IFERROR(VLOOKUP(J5,Fiat!$B$1:$C$20,2,FALSE)*K5,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
-      <c r="M5" s="32" t="str" cm="1">
+      <c r="M5" s="17" t="str" cm="1">
         <f t="array" ref="M5">IFERROR((_FV(C5,"Price")-_FV(C5,"52 week low",TRUE))/(_FV(C5,"52 week high",TRUE)-_FV(C5,"52 week low",TRUE)),"")</f>
         <v/>
       </c>
@@ -1916,7 +1819,7 @@
         <f>IF(K6="","",IFERROR(VLOOKUP(J6,Fiat!$B$1:$C$20,2,FALSE)*K6,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
-      <c r="M6" s="32" t="str" cm="1">
+      <c r="M6" s="17" t="str" cm="1">
         <f t="array" ref="M6">IFERROR((_FV(C6,"Price")-_FV(C6,"52 week low",TRUE))/(_FV(C6,"52 week high",TRUE)-_FV(C6,"52 week low",TRUE)),"")</f>
         <v/>
       </c>
@@ -1953,7 +1856,7 @@
         <f>IF(K7="","",IFERROR(VLOOKUP(J7,Fiat!$B$1:$C$20,2,FALSE)*K7,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
-      <c r="M7" s="32" t="str" cm="1">
+      <c r="M7" s="17" t="str" cm="1">
         <f t="array" ref="M7">IFERROR((_FV(C7,"Price")-_FV(C7,"52 week low",TRUE))/(_FV(C7,"52 week high",TRUE)-_FV(C7,"52 week low",TRUE)),"")</f>
         <v/>
       </c>
@@ -1989,7 +1892,7 @@
         <f>IF(K8="","",IFERROR(VLOOKUP(J8,Fiat!$B$1:$C$20,2,FALSE)*K8,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
-      <c r="M8" s="32" t="str" cm="1">
+      <c r="M8" s="17" t="str" cm="1">
         <f t="array" ref="M8">IFERROR((_FV(C8,"Price")-_FV(C8,"52 week low",TRUE))/(_FV(C8,"52 week high",TRUE)-_FV(C8,"52 week low",TRUE)),"")</f>
         <v/>
       </c>
@@ -2026,7 +1929,7 @@
         <f>IF(K9="","",IFERROR(VLOOKUP(J9,Fiat!$B$1:$C$20,2,FALSE)*K9,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
-      <c r="M9" s="32" t="str" cm="1">
+      <c r="M9" s="17" t="str" cm="1">
         <f t="array" ref="M9">IFERROR((_FV(C9,"Price")-_FV(C9,"52 week low",TRUE))/(_FV(C9,"52 week high",TRUE)-_FV(C9,"52 week low",TRUE)),"")</f>
         <v/>
       </c>
@@ -2057,7 +1960,7 @@
         <f>IF(K10="","",IFERROR(VLOOKUP(J10,Fiat!$B$1:$C$20,2,FALSE)*K10,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
-      <c r="M10" s="32" t="str" cm="1">
+      <c r="M10" s="17" t="str" cm="1">
         <f t="array" ref="M10">IFERROR((_FV(C10,"Price")-_FV(C10,"52 week low",TRUE))/(_FV(C10,"52 week high",TRUE)-_FV(C10,"52 week low",TRUE)),"")</f>
         <v/>
       </c>
@@ -2075,15 +1978,15 @@
         <f t="array" ref="J11">IFERROR(_FV(C11,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K11" s="30" t="str" cm="1">
+      <c r="K11" s="24" t="str" cm="1">
         <f t="array" ref="K11">IFERROR(_FV(C11,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L11" s="30" t="str">
+      <c r="L11" s="24" t="str">
         <f>IF(K11="","",IFERROR(VLOOKUP(J11,Fiat!$B$1:$C$20,2,FALSE)*K11,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
-      <c r="M11" s="33" t="str" cm="1">
+      <c r="M11" s="26" t="str" cm="1">
         <f t="array" ref="M11">IFERROR((_FV(C11,"Price")-_FV(C11,"52 week low",TRUE))/(_FV(C11,"52 week high",TRUE)-_FV(C11,"52 week low",TRUE)),"")</f>
         <v/>
       </c>
@@ -2101,15 +2004,15 @@
         <f t="array" ref="J12">IFERROR(_FV(C12,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K12" s="30" t="str" cm="1">
+      <c r="K12" s="24" t="str" cm="1">
         <f t="array" ref="K12">IFERROR(_FV(C12,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L12" s="30" t="str">
+      <c r="L12" s="24" t="str">
         <f>IF(K12="","",IFERROR(VLOOKUP(J12,Fiat!$B$1:$C$20,2,FALSE)*K12,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
-      <c r="M12" s="33" t="str" cm="1">
+      <c r="M12" s="26" t="str" cm="1">
         <f t="array" ref="M12">IFERROR((_FV(C12,"Price")-_FV(C12,"52 week low",TRUE))/(_FV(C12,"52 week high",TRUE)-_FV(C12,"52 week low",TRUE)),"")</f>
         <v/>
       </c>
@@ -2127,15 +2030,15 @@
         <f t="array" ref="J13">IFERROR(_FV(C13,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K13" s="30" t="str" cm="1">
+      <c r="K13" s="24" t="str" cm="1">
         <f t="array" ref="K13">IFERROR(_FV(C13,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L13" s="30" t="str">
+      <c r="L13" s="24" t="str">
         <f>IF(K13="","",IFERROR(VLOOKUP(J13,Fiat!$B$1:$C$20,2,FALSE)*K13,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
-      <c r="M13" s="33" t="str" cm="1">
+      <c r="M13" s="26" t="str" cm="1">
         <f t="array" ref="M13">IFERROR((_FV(C13,"Price")-_FV(C13,"52 week low",TRUE))/(_FV(C13,"52 week high",TRUE)-_FV(C13,"52 week low",TRUE)),"")</f>
         <v/>
       </c>
@@ -2420,11 +2323,11 @@
         <f t="array" ref="J21">IFERROR(_FV(C21,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K21" s="31" t="str" cm="1">
+      <c r="K21" s="25" t="str" cm="1">
         <f t="array" ref="K21">IFERROR(_FV(C21,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L21" s="31" t="str">
+      <c r="L21" s="25" t="str">
         <f>IF(K21="","",IFERROR(VLOOKUP(J21,Fiat!$B$1:$C$20,2,FALSE)*K21,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2457,11 +2360,11 @@
         <f t="array" ref="J22">IFERROR(_FV(C22,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K22" s="31" t="str" cm="1">
+      <c r="K22" s="25" t="str" cm="1">
         <f t="array" ref="K22">IFERROR(_FV(C22,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L22" s="31" t="str">
+      <c r="L22" s="25" t="str">
         <f>IF(K22="","",IFERROR(VLOOKUP(J22,Fiat!$B$1:$C$20,2,FALSE)*K22,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2494,11 +2397,11 @@
         <f t="array" ref="J23">IFERROR(_FV(C23,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K23" s="31" t="str" cm="1">
+      <c r="K23" s="25" t="str" cm="1">
         <f t="array" ref="K23">IFERROR(_FV(C23,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L23" s="31" t="str">
+      <c r="L23" s="25" t="str">
         <f>IF(K23="","",IFERROR(VLOOKUP(J23,Fiat!$B$1:$C$20,2,FALSE)*K23,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2531,11 +2434,11 @@
         <f t="array" ref="J24">IFERROR(_FV(C24,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K24" s="31" t="str" cm="1">
+      <c r="K24" s="25" t="str" cm="1">
         <f t="array" ref="K24">IFERROR(_FV(C24,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L24" s="31" t="str">
+      <c r="L24" s="25" t="str">
         <f>IF(K24="","",IFERROR(VLOOKUP(J24,Fiat!$B$1:$C$20,2,FALSE)*K24,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2568,11 +2471,11 @@
         <f t="array" ref="J25">IFERROR(_FV(C25,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K25" s="31" t="str" cm="1">
+      <c r="K25" s="25" t="str" cm="1">
         <f t="array" ref="K25">IFERROR(_FV(C25,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L25" s="31" t="str">
+      <c r="L25" s="25" t="str">
         <f>IF(K25="","",IFERROR(VLOOKUP(J25,Fiat!$B$1:$C$20,2,FALSE)*K25,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2605,11 +2508,11 @@
         <f t="array" ref="J26">IFERROR(_FV(C26,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K26" s="31" t="str" cm="1">
+      <c r="K26" s="25" t="str" cm="1">
         <f t="array" ref="K26">IFERROR(_FV(C26,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L26" s="31" t="str">
+      <c r="L26" s="25" t="str">
         <f>IF(K26="","",IFERROR(VLOOKUP(J26,Fiat!$B$1:$C$20,2,FALSE)*K26,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2642,11 +2545,11 @@
         <f t="array" ref="J27">IFERROR(_FV(C27,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K27" s="31" t="str" cm="1">
+      <c r="K27" s="25" t="str" cm="1">
         <f t="array" ref="K27">IFERROR(_FV(C27,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L27" s="31" t="str">
+      <c r="L27" s="25" t="str">
         <f>IF(K27="","",IFERROR(VLOOKUP(J27,Fiat!$B$1:$C$20,2,FALSE)*K27,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2679,11 +2582,11 @@
         <f t="array" ref="J28">IFERROR(_FV(C28,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K28" s="31" t="str" cm="1">
+      <c r="K28" s="25" t="str" cm="1">
         <f t="array" ref="K28">IFERROR(_FV(C28,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L28" s="31" t="str">
+      <c r="L28" s="25" t="str">
         <f>IF(K28="","",IFERROR(VLOOKUP(J28,Fiat!$B$1:$C$20,2,FALSE)*K28,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2716,11 +2619,11 @@
         <f t="array" ref="J29">IFERROR(_FV(C29,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K29" s="31" t="str" cm="1">
+      <c r="K29" s="25" t="str" cm="1">
         <f t="array" ref="K29">IFERROR(_FV(C29,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L29" s="31" t="str">
+      <c r="L29" s="25" t="str">
         <f>IF(K29="","",IFERROR(VLOOKUP(J29,Fiat!$B$1:$C$20,2,FALSE)*K29,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2753,11 +2656,11 @@
         <f t="array" ref="J30">IFERROR(_FV(C30,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K30" s="31" t="str" cm="1">
+      <c r="K30" s="25" t="str" cm="1">
         <f t="array" ref="K30">IFERROR(_FV(C30,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L30" s="31" t="str">
+      <c r="L30" s="25" t="str">
         <f>IF(K30="","",IFERROR(VLOOKUP(J30,Fiat!$B$1:$C$20,2,FALSE)*K30,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2790,11 +2693,11 @@
         <f t="array" ref="J31">IFERROR(_FV(C31,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K31" s="31" t="str" cm="1">
+      <c r="K31" s="25" t="str" cm="1">
         <f t="array" ref="K31">IFERROR(_FV(C31,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L31" s="31" t="str">
+      <c r="L31" s="25" t="str">
         <f>IF(K31="","",IFERROR(VLOOKUP(J31,Fiat!$B$1:$C$20,2,FALSE)*K31,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2827,11 +2730,11 @@
         <f t="array" ref="J32">IFERROR(_FV(C32,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K32" s="31" t="str" cm="1">
+      <c r="K32" s="25" t="str" cm="1">
         <f t="array" ref="K32">IFERROR(_FV(C32,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L32" s="31" t="str">
+      <c r="L32" s="25" t="str">
         <f>IF(K32="","",IFERROR(VLOOKUP(J32,Fiat!$B$1:$C$20,2,FALSE)*K32,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2864,11 +2767,11 @@
         <f t="array" ref="J33">IFERROR(_FV(C33,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K33" s="31" t="str" cm="1">
+      <c r="K33" s="25" t="str" cm="1">
         <f t="array" ref="K33">IFERROR(_FV(C33,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L33" s="31" t="str">
+      <c r="L33" s="25" t="str">
         <f>IF(K33="","",IFERROR(VLOOKUP(J33,Fiat!$B$1:$C$20,2,FALSE)*K33,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2901,11 +2804,11 @@
         <f t="array" ref="J34">IFERROR(_FV(C34,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K34" s="31" t="str" cm="1">
+      <c r="K34" s="25" t="str" cm="1">
         <f t="array" ref="K34">IFERROR(_FV(C34,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L34" s="31" t="str">
+      <c r="L34" s="25" t="str">
         <f>IF(K34="","",IFERROR(VLOOKUP(J34,Fiat!$B$1:$C$20,2,FALSE)*K34,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2938,11 +2841,11 @@
         <f t="array" ref="J35">IFERROR(_FV(C35,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K35" s="31" t="str" cm="1">
+      <c r="K35" s="25" t="str" cm="1">
         <f t="array" ref="K35">IFERROR(_FV(C35,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L35" s="31" t="str">
+      <c r="L35" s="25" t="str">
         <f>IF(K35="","",IFERROR(VLOOKUP(J35,Fiat!$B$1:$C$20,2,FALSE)*K35,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -2975,11 +2878,11 @@
         <f t="array" ref="J36">IFERROR(_FV(C36,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K36" s="31" t="str" cm="1">
+      <c r="K36" s="25" t="str" cm="1">
         <f t="array" ref="K36">IFERROR(_FV(C36,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L36" s="31" t="str">
+      <c r="L36" s="25" t="str">
         <f>IF(K36="","",IFERROR(VLOOKUP(J36,Fiat!$B$1:$C$20,2,FALSE)*K36,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3012,11 +2915,11 @@
         <f t="array" ref="J37">IFERROR(_FV(C37,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K37" s="31" t="str" cm="1">
+      <c r="K37" s="25" t="str" cm="1">
         <f t="array" ref="K37">IFERROR(_FV(C37,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L37" s="31" t="str">
+      <c r="L37" s="25" t="str">
         <f>IF(K37="","",IFERROR(VLOOKUP(J37,Fiat!$B$1:$C$20,2,FALSE)*K37,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3049,11 +2952,11 @@
         <f t="array" ref="J38">IFERROR(_FV(C38,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K38" s="31" t="str" cm="1">
+      <c r="K38" s="25" t="str" cm="1">
         <f t="array" ref="K38">IFERROR(_FV(C38,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L38" s="31" t="str">
+      <c r="L38" s="25" t="str">
         <f>IF(K38="","",IFERROR(VLOOKUP(J38,Fiat!$B$1:$C$20,2,FALSE)*K38,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3086,11 +2989,11 @@
         <f t="array" ref="J39">IFERROR(_FV(C39,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K39" s="31" t="str" cm="1">
+      <c r="K39" s="25" t="str" cm="1">
         <f t="array" ref="K39">IFERROR(_FV(C39,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L39" s="31" t="str">
+      <c r="L39" s="25" t="str">
         <f>IF(K39="","",IFERROR(VLOOKUP(J39,Fiat!$B$1:$C$20,2,FALSE)*K39,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3123,11 +3026,11 @@
         <f t="array" ref="J40">IFERROR(_FV(C40,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K40" s="31" t="str" cm="1">
+      <c r="K40" s="25" t="str" cm="1">
         <f t="array" ref="K40">IFERROR(_FV(C40,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L40" s="31" t="str">
+      <c r="L40" s="25" t="str">
         <f>IF(K40="","",IFERROR(VLOOKUP(J40,Fiat!$B$1:$C$20,2,FALSE)*K40,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3160,11 +3063,11 @@
         <f t="array" ref="J41">IFERROR(_FV(C41,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K41" s="31" t="str" cm="1">
+      <c r="K41" s="25" t="str" cm="1">
         <f t="array" ref="K41">IFERROR(_FV(C41,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L41" s="31" t="str">
+      <c r="L41" s="25" t="str">
         <f>IF(K41="","",IFERROR(VLOOKUP(J41,Fiat!$B$1:$C$20,2,FALSE)*K41,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3197,11 +3100,11 @@
         <f t="array" ref="J42">IFERROR(_FV(C42,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K42" s="31" t="str" cm="1">
+      <c r="K42" s="25" t="str" cm="1">
         <f t="array" ref="K42">IFERROR(_FV(C42,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L42" s="31" t="str">
+      <c r="L42" s="25" t="str">
         <f>IF(K42="","",IFERROR(VLOOKUP(J42,Fiat!$B$1:$C$20,2,FALSE)*K42,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3234,11 +3137,11 @@
         <f t="array" ref="J43">IFERROR(_FV(C43,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K43" s="31" t="str" cm="1">
+      <c r="K43" s="25" t="str" cm="1">
         <f t="array" ref="K43">IFERROR(_FV(C43,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L43" s="31" t="str">
+      <c r="L43" s="25" t="str">
         <f>IF(K43="","",IFERROR(VLOOKUP(J43,Fiat!$B$1:$C$20,2,FALSE)*K43,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3271,11 +3174,11 @@
         <f t="array" ref="J44">IFERROR(_FV(C44,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K44" s="31" t="str" cm="1">
+      <c r="K44" s="25" t="str" cm="1">
         <f t="array" ref="K44">IFERROR(_FV(C44,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L44" s="31" t="str">
+      <c r="L44" s="25" t="str">
         <f>IF(K44="","",IFERROR(VLOOKUP(J44,Fiat!$B$1:$C$20,2,FALSE)*K44,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3308,11 +3211,11 @@
         <f t="array" ref="J45">IFERROR(_FV(C45,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K45" s="31" t="str" cm="1">
+      <c r="K45" s="25" t="str" cm="1">
         <f t="array" ref="K45">IFERROR(_FV(C45,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L45" s="31" t="str">
+      <c r="L45" s="25" t="str">
         <f>IF(K45="","",IFERROR(VLOOKUP(J45,Fiat!$B$1:$C$20,2,FALSE)*K45,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3345,11 +3248,11 @@
         <f t="array" ref="J46">IFERROR(_FV(C46,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K46" s="31" t="str" cm="1">
+      <c r="K46" s="25" t="str" cm="1">
         <f t="array" ref="K46">IFERROR(_FV(C46,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L46" s="31" t="str">
+      <c r="L46" s="25" t="str">
         <f>IF(K46="","",IFERROR(VLOOKUP(J46,Fiat!$B$1:$C$20,2,FALSE)*K46,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3382,11 +3285,11 @@
         <f t="array" ref="J47">IFERROR(_FV(C47,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K47" s="31" t="str" cm="1">
+      <c r="K47" s="25" t="str" cm="1">
         <f t="array" ref="K47">IFERROR(_FV(C47,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L47" s="31" t="str">
+      <c r="L47" s="25" t="str">
         <f>IF(K47="","",IFERROR(VLOOKUP(J47,Fiat!$B$1:$C$20,2,FALSE)*K47,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3419,11 +3322,11 @@
         <f t="array" ref="J48">IFERROR(_FV(C48,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K48" s="31" t="str" cm="1">
+      <c r="K48" s="25" t="str" cm="1">
         <f t="array" ref="K48">IFERROR(_FV(C48,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L48" s="31" t="str">
+      <c r="L48" s="25" t="str">
         <f>IF(K48="","",IFERROR(VLOOKUP(J48,Fiat!$B$1:$C$20,2,FALSE)*K48,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3456,11 +3359,11 @@
         <f t="array" ref="J49">IFERROR(_FV(C49,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K49" s="31" t="str" cm="1">
+      <c r="K49" s="25" t="str" cm="1">
         <f t="array" ref="K49">IFERROR(_FV(C49,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L49" s="31" t="str">
+      <c r="L49" s="25" t="str">
         <f>IF(K49="","",IFERROR(VLOOKUP(J49,Fiat!$B$1:$C$20,2,FALSE)*K49,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3493,11 +3396,11 @@
         <f t="array" ref="J50">IFERROR(_FV(C50,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K50" s="31" t="str" cm="1">
+      <c r="K50" s="25" t="str" cm="1">
         <f t="array" ref="K50">IFERROR(_FV(C50,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L50" s="31" t="str">
+      <c r="L50" s="25" t="str">
         <f>IF(K50="","",IFERROR(VLOOKUP(J50,Fiat!$B$1:$C$20,2,FALSE)*K50,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3530,11 +3433,11 @@
         <f t="array" ref="J51">IFERROR(_FV(C51,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K51" s="31" t="str" cm="1">
+      <c r="K51" s="25" t="str" cm="1">
         <f t="array" ref="K51">IFERROR(_FV(C51,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L51" s="31" t="str">
+      <c r="L51" s="25" t="str">
         <f>IF(K51="","",IFERROR(VLOOKUP(J51,Fiat!$B$1:$C$20,2,FALSE)*K51,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3567,11 +3470,11 @@
         <f t="array" ref="J52">IFERROR(_FV(C52,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K52" s="31" t="str" cm="1">
+      <c r="K52" s="25" t="str" cm="1">
         <f t="array" ref="K52">IFERROR(_FV(C52,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L52" s="31" t="str">
+      <c r="L52" s="25" t="str">
         <f>IF(K52="","",IFERROR(VLOOKUP(J52,Fiat!$B$1:$C$20,2,FALSE)*K52,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3604,11 +3507,11 @@
         <f t="array" ref="J53">IFERROR(_FV(C53,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K53" s="31" t="str" cm="1">
+      <c r="K53" s="25" t="str" cm="1">
         <f t="array" ref="K53">IFERROR(_FV(C53,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L53" s="31" t="str">
+      <c r="L53" s="25" t="str">
         <f>IF(K53="","",IFERROR(VLOOKUP(J53,Fiat!$B$1:$C$20,2,FALSE)*K53,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3641,11 +3544,11 @@
         <f t="array" ref="J54">IFERROR(_FV(C54,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K54" s="31" t="str" cm="1">
+      <c r="K54" s="25" t="str" cm="1">
         <f t="array" ref="K54">IFERROR(_FV(C54,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L54" s="31" t="str">
+      <c r="L54" s="25" t="str">
         <f>IF(K54="","",IFERROR(VLOOKUP(J54,Fiat!$B$1:$C$20,2,FALSE)*K54,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3678,11 +3581,11 @@
         <f t="array" ref="J55">IFERROR(_FV(C55,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K55" s="31" t="str" cm="1">
+      <c r="K55" s="25" t="str" cm="1">
         <f t="array" ref="K55">IFERROR(_FV(C55,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L55" s="31" t="str">
+      <c r="L55" s="25" t="str">
         <f>IF(K55="","",IFERROR(VLOOKUP(J55,Fiat!$B$1:$C$20,2,FALSE)*K55,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3715,11 +3618,11 @@
         <f t="array" ref="J56">IFERROR(_FV(C56,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K56" s="31" t="str" cm="1">
+      <c r="K56" s="25" t="str" cm="1">
         <f t="array" ref="K56">IFERROR(_FV(C56,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L56" s="31" t="str">
+      <c r="L56" s="25" t="str">
         <f>IF(K56="","",IFERROR(VLOOKUP(J56,Fiat!$B$1:$C$20,2,FALSE)*K56,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3752,11 +3655,11 @@
         <f t="array" ref="J57">IFERROR(_FV(C57,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K57" s="31" t="str" cm="1">
+      <c r="K57" s="25" t="str" cm="1">
         <f t="array" ref="K57">IFERROR(_FV(C57,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L57" s="31" t="str">
+      <c r="L57" s="25" t="str">
         <f>IF(K57="","",IFERROR(VLOOKUP(J57,Fiat!$B$1:$C$20,2,FALSE)*K57,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3789,11 +3692,11 @@
         <f t="array" ref="J58">IFERROR(_FV(C58,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K58" s="31" t="str" cm="1">
+      <c r="K58" s="25" t="str" cm="1">
         <f t="array" ref="K58">IFERROR(_FV(C58,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L58" s="31" t="str">
+      <c r="L58" s="25" t="str">
         <f>IF(K58="","",IFERROR(VLOOKUP(J58,Fiat!$B$1:$C$20,2,FALSE)*K58,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3826,11 +3729,11 @@
         <f t="array" ref="J59">IFERROR(_FV(C59,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K59" s="31" t="str" cm="1">
+      <c r="K59" s="25" t="str" cm="1">
         <f t="array" ref="K59">IFERROR(_FV(C59,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L59" s="31" t="str">
+      <c r="L59" s="25" t="str">
         <f>IF(K59="","",IFERROR(VLOOKUP(J59,Fiat!$B$1:$C$20,2,FALSE)*K59,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3863,11 +3766,11 @@
         <f t="array" ref="J60">IFERROR(_FV(C60,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K60" s="31" t="str" cm="1">
+      <c r="K60" s="25" t="str" cm="1">
         <f t="array" ref="K60">IFERROR(_FV(C60,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L60" s="31" t="str">
+      <c r="L60" s="25" t="str">
         <f>IF(K60="","",IFERROR(VLOOKUP(J60,Fiat!$B$1:$C$20,2,FALSE)*K60,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3900,11 +3803,11 @@
         <f t="array" ref="J61">IFERROR(_FV(C61,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K61" s="31" t="str" cm="1">
+      <c r="K61" s="25" t="str" cm="1">
         <f t="array" ref="K61">IFERROR(_FV(C61,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L61" s="31" t="str">
+      <c r="L61" s="25" t="str">
         <f>IF(K61="","",IFERROR(VLOOKUP(J61,Fiat!$B$1:$C$20,2,FALSE)*K61,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3937,11 +3840,11 @@
         <f t="array" ref="J62">IFERROR(_FV(C62,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K62" s="31" t="str" cm="1">
+      <c r="K62" s="25" t="str" cm="1">
         <f t="array" ref="K62">IFERROR(_FV(C62,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L62" s="31" t="str">
+      <c r="L62" s="25" t="str">
         <f>IF(K62="","",IFERROR(VLOOKUP(J62,Fiat!$B$1:$C$20,2,FALSE)*K62,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -3974,11 +3877,11 @@
         <f t="array" ref="J63">IFERROR(_FV(C63,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K63" s="31" t="str" cm="1">
+      <c r="K63" s="25" t="str" cm="1">
         <f t="array" ref="K63">IFERROR(_FV(C63,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L63" s="31" t="str">
+      <c r="L63" s="25" t="str">
         <f>IF(K63="","",IFERROR(VLOOKUP(J63,Fiat!$B$1:$C$20,2,FALSE)*K63,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4011,11 +3914,11 @@
         <f t="array" ref="J64">IFERROR(_FV(C64,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K64" s="31" t="str" cm="1">
+      <c r="K64" s="25" t="str" cm="1">
         <f t="array" ref="K64">IFERROR(_FV(C64,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L64" s="31" t="str">
+      <c r="L64" s="25" t="str">
         <f>IF(K64="","",IFERROR(VLOOKUP(J64,Fiat!$B$1:$C$20,2,FALSE)*K64,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4048,11 +3951,11 @@
         <f t="array" ref="J65">IFERROR(_FV(C65,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K65" s="31" t="str" cm="1">
+      <c r="K65" s="25" t="str" cm="1">
         <f t="array" ref="K65">IFERROR(_FV(C65,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L65" s="31" t="str">
+      <c r="L65" s="25" t="str">
         <f>IF(K65="","",IFERROR(VLOOKUP(J65,Fiat!$B$1:$C$20,2,FALSE)*K65,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4085,11 +3988,11 @@
         <f t="array" ref="J66">IFERROR(_FV(C66,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K66" s="31" t="str" cm="1">
+      <c r="K66" s="25" t="str" cm="1">
         <f t="array" ref="K66">IFERROR(_FV(C66,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L66" s="31" t="str">
+      <c r="L66" s="25" t="str">
         <f>IF(K66="","",IFERROR(VLOOKUP(J66,Fiat!$B$1:$C$20,2,FALSE)*K66,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4122,11 +4025,11 @@
         <f t="array" ref="J67">IFERROR(_FV(C67,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K67" s="31" t="str" cm="1">
+      <c r="K67" s="25" t="str" cm="1">
         <f t="array" ref="K67">IFERROR(_FV(C67,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L67" s="31" t="str">
+      <c r="L67" s="25" t="str">
         <f>IF(K67="","",IFERROR(VLOOKUP(J67,Fiat!$B$1:$C$20,2,FALSE)*K67,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4159,11 +4062,11 @@
         <f t="array" ref="J68">IFERROR(_FV(C68,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K68" s="31" t="str" cm="1">
+      <c r="K68" s="25" t="str" cm="1">
         <f t="array" ref="K68">IFERROR(_FV(C68,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L68" s="31" t="str">
+      <c r="L68" s="25" t="str">
         <f>IF(K68="","",IFERROR(VLOOKUP(J68,Fiat!$B$1:$C$20,2,FALSE)*K68,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4196,11 +4099,11 @@
         <f t="array" ref="J69">IFERROR(_FV(C69,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K69" s="31" t="str" cm="1">
+      <c r="K69" s="25" t="str" cm="1">
         <f t="array" ref="K69">IFERROR(_FV(C69,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L69" s="31" t="str">
+      <c r="L69" s="25" t="str">
         <f>IF(K69="","",IFERROR(VLOOKUP(J69,Fiat!$B$1:$C$20,2,FALSE)*K69,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4233,11 +4136,11 @@
         <f t="array" ref="J70">IFERROR(_FV(C70,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K70" s="31" t="str" cm="1">
+      <c r="K70" s="25" t="str" cm="1">
         <f t="array" ref="K70">IFERROR(_FV(C70,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L70" s="31" t="str">
+      <c r="L70" s="25" t="str">
         <f>IF(K70="","",IFERROR(VLOOKUP(J70,Fiat!$B$1:$C$20,2,FALSE)*K70,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4270,11 +4173,11 @@
         <f t="array" ref="J71">IFERROR(_FV(C71,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K71" s="31" t="str" cm="1">
+      <c r="K71" s="25" t="str" cm="1">
         <f t="array" ref="K71">IFERROR(_FV(C71,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L71" s="31" t="str">
+      <c r="L71" s="25" t="str">
         <f>IF(K71="","",IFERROR(VLOOKUP(J71,Fiat!$B$1:$C$20,2,FALSE)*K71,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4307,11 +4210,11 @@
         <f t="array" ref="J72">IFERROR(_FV(C72,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K72" s="31" t="str" cm="1">
+      <c r="K72" s="25" t="str" cm="1">
         <f t="array" ref="K72">IFERROR(_FV(C72,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L72" s="31" t="str">
+      <c r="L72" s="25" t="str">
         <f>IF(K72="","",IFERROR(VLOOKUP(J72,Fiat!$B$1:$C$20,2,FALSE)*K72,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4344,11 +4247,11 @@
         <f t="array" ref="J73">IFERROR(_FV(C73,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K73" s="31" t="str" cm="1">
+      <c r="K73" s="25" t="str" cm="1">
         <f t="array" ref="K73">IFERROR(_FV(C73,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L73" s="31" t="str">
+      <c r="L73" s="25" t="str">
         <f>IF(K73="","",IFERROR(VLOOKUP(J73,Fiat!$B$1:$C$20,2,FALSE)*K73,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4381,11 +4284,11 @@
         <f t="array" ref="J74">IFERROR(_FV(C74,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K74" s="31" t="str" cm="1">
+      <c r="K74" s="25" t="str" cm="1">
         <f t="array" ref="K74">IFERROR(_FV(C74,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L74" s="31" t="str">
+      <c r="L74" s="25" t="str">
         <f>IF(K74="","",IFERROR(VLOOKUP(J74,Fiat!$B$1:$C$20,2,FALSE)*K74,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4418,11 +4321,11 @@
         <f t="array" ref="J75">IFERROR(_FV(C75,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K75" s="31" t="str" cm="1">
+      <c r="K75" s="25" t="str" cm="1">
         <f t="array" ref="K75">IFERROR(_FV(C75,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L75" s="31" t="str">
+      <c r="L75" s="25" t="str">
         <f>IF(K75="","",IFERROR(VLOOKUP(J75,Fiat!$B$1:$C$20,2,FALSE)*K75,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4455,11 +4358,11 @@
         <f t="array" ref="J76">IFERROR(_FV(C76,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K76" s="31" t="str" cm="1">
+      <c r="K76" s="25" t="str" cm="1">
         <f t="array" ref="K76">IFERROR(_FV(C76,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L76" s="31" t="str">
+      <c r="L76" s="25" t="str">
         <f>IF(K76="","",IFERROR(VLOOKUP(J76,Fiat!$B$1:$C$20,2,FALSE)*K76,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4492,11 +4395,11 @@
         <f t="array" ref="J77">IFERROR(_FV(C77,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K77" s="31" t="str" cm="1">
+      <c r="K77" s="25" t="str" cm="1">
         <f t="array" ref="K77">IFERROR(_FV(C77,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L77" s="31" t="str">
+      <c r="L77" s="25" t="str">
         <f>IF(K77="","",IFERROR(VLOOKUP(J77,Fiat!$B$1:$C$20,2,FALSE)*K77,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4529,11 +4432,11 @@
         <f t="array" ref="J78">IFERROR(_FV(C78,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K78" s="31" t="str" cm="1">
+      <c r="K78" s="25" t="str" cm="1">
         <f t="array" ref="K78">IFERROR(_FV(C78,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L78" s="31" t="str">
+      <c r="L78" s="25" t="str">
         <f>IF(K78="","",IFERROR(VLOOKUP(J78,Fiat!$B$1:$C$20,2,FALSE)*K78,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4566,11 +4469,11 @@
         <f t="array" ref="J79">IFERROR(_FV(C79,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K79" s="31" t="str" cm="1">
+      <c r="K79" s="25" t="str" cm="1">
         <f t="array" ref="K79">IFERROR(_FV(C79,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L79" s="31" t="str">
+      <c r="L79" s="25" t="str">
         <f>IF(K79="","",IFERROR(VLOOKUP(J79,Fiat!$B$1:$C$20,2,FALSE)*K79,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4603,11 +4506,11 @@
         <f t="array" ref="J80">IFERROR(_FV(C80,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K80" s="31" t="str" cm="1">
+      <c r="K80" s="25" t="str" cm="1">
         <f t="array" ref="K80">IFERROR(_FV(C80,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L80" s="31" t="str">
+      <c r="L80" s="25" t="str">
         <f>IF(K80="","",IFERROR(VLOOKUP(J80,Fiat!$B$1:$C$20,2,FALSE)*K80,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4640,11 +4543,11 @@
         <f t="array" ref="J81">IFERROR(_FV(C81,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K81" s="31" t="str" cm="1">
+      <c r="K81" s="25" t="str" cm="1">
         <f t="array" ref="K81">IFERROR(_FV(C81,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L81" s="31" t="str">
+      <c r="L81" s="25" t="str">
         <f>IF(K81="","",IFERROR(VLOOKUP(J81,Fiat!$B$1:$C$20,2,FALSE)*K81,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4677,11 +4580,11 @@
         <f t="array" ref="J82">IFERROR(_FV(C82,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K82" s="31" t="str" cm="1">
+      <c r="K82" s="25" t="str" cm="1">
         <f t="array" ref="K82">IFERROR(_FV(C82,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L82" s="31" t="str">
+      <c r="L82" s="25" t="str">
         <f>IF(K82="","",IFERROR(VLOOKUP(J82,Fiat!$B$1:$C$20,2,FALSE)*K82,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4714,11 +4617,11 @@
         <f t="array" ref="J83">IFERROR(_FV(C83,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K83" s="31" t="str" cm="1">
+      <c r="K83" s="25" t="str" cm="1">
         <f t="array" ref="K83">IFERROR(_FV(C83,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L83" s="31" t="str">
+      <c r="L83" s="25" t="str">
         <f>IF(K83="","",IFERROR(VLOOKUP(J83,Fiat!$B$1:$C$20,2,FALSE)*K83,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4751,11 +4654,11 @@
         <f t="array" ref="J84">IFERROR(_FV(C84,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K84" s="31" t="str" cm="1">
+      <c r="K84" s="25" t="str" cm="1">
         <f t="array" ref="K84">IFERROR(_FV(C84,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L84" s="31" t="str">
+      <c r="L84" s="25" t="str">
         <f>IF(K84="","",IFERROR(VLOOKUP(J84,Fiat!$B$1:$C$20,2,FALSE)*K84,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4788,11 +4691,11 @@
         <f t="array" ref="J85">IFERROR(_FV(C85,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K85" s="31" t="str" cm="1">
+      <c r="K85" s="25" t="str" cm="1">
         <f t="array" ref="K85">IFERROR(_FV(C85,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L85" s="31" t="str">
+      <c r="L85" s="25" t="str">
         <f>IF(K85="","",IFERROR(VLOOKUP(J85,Fiat!$B$1:$C$20,2,FALSE)*K85,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4825,11 +4728,11 @@
         <f t="array" ref="J86">IFERROR(_FV(C86,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K86" s="31" t="str" cm="1">
+      <c r="K86" s="25" t="str" cm="1">
         <f t="array" ref="K86">IFERROR(_FV(C86,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L86" s="31" t="str">
+      <c r="L86" s="25" t="str">
         <f>IF(K86="","",IFERROR(VLOOKUP(J86,Fiat!$B$1:$C$20,2,FALSE)*K86,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4862,11 +4765,11 @@
         <f t="array" ref="J87">IFERROR(_FV(C87,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K87" s="31" t="str" cm="1">
+      <c r="K87" s="25" t="str" cm="1">
         <f t="array" ref="K87">IFERROR(_FV(C87,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L87" s="31" t="str">
+      <c r="L87" s="25" t="str">
         <f>IF(K87="","",IFERROR(VLOOKUP(J87,Fiat!$B$1:$C$20,2,FALSE)*K87,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4899,11 +4802,11 @@
         <f t="array" ref="J88">IFERROR(_FV(C88,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K88" s="31" t="str" cm="1">
+      <c r="K88" s="25" t="str" cm="1">
         <f t="array" ref="K88">IFERROR(_FV(C88,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L88" s="31" t="str">
+      <c r="L88" s="25" t="str">
         <f>IF(K88="","",IFERROR(VLOOKUP(J88,Fiat!$B$1:$C$20,2,FALSE)*K88,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4936,11 +4839,11 @@
         <f t="array" ref="J89">IFERROR(_FV(C89,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K89" s="31" t="str" cm="1">
+      <c r="K89" s="25" t="str" cm="1">
         <f t="array" ref="K89">IFERROR(_FV(C89,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L89" s="31" t="str">
+      <c r="L89" s="25" t="str">
         <f>IF(K89="","",IFERROR(VLOOKUP(J89,Fiat!$B$1:$C$20,2,FALSE)*K89,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -4973,11 +4876,11 @@
         <f t="array" ref="J90">IFERROR(_FV(C90,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K90" s="31" t="str" cm="1">
+      <c r="K90" s="25" t="str" cm="1">
         <f t="array" ref="K90">IFERROR(_FV(C90,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L90" s="31" t="str">
+      <c r="L90" s="25" t="str">
         <f>IF(K90="","",IFERROR(VLOOKUP(J90,Fiat!$B$1:$C$20,2,FALSE)*K90,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5010,11 +4913,11 @@
         <f t="array" ref="J91">IFERROR(_FV(C91,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K91" s="31" t="str" cm="1">
+      <c r="K91" s="25" t="str" cm="1">
         <f t="array" ref="K91">IFERROR(_FV(C91,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L91" s="31" t="str">
+      <c r="L91" s="25" t="str">
         <f>IF(K91="","",IFERROR(VLOOKUP(J91,Fiat!$B$1:$C$20,2,FALSE)*K91,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5047,11 +4950,11 @@
         <f t="array" ref="J92">IFERROR(_FV(C92,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K92" s="31" t="str" cm="1">
+      <c r="K92" s="25" t="str" cm="1">
         <f t="array" ref="K92">IFERROR(_FV(C92,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L92" s="31" t="str">
+      <c r="L92" s="25" t="str">
         <f>IF(K92="","",IFERROR(VLOOKUP(J92,Fiat!$B$1:$C$20,2,FALSE)*K92,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5084,11 +4987,11 @@
         <f t="array" ref="J93">IFERROR(_FV(C93,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K93" s="31" t="str" cm="1">
+      <c r="K93" s="25" t="str" cm="1">
         <f t="array" ref="K93">IFERROR(_FV(C93,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L93" s="31" t="str">
+      <c r="L93" s="25" t="str">
         <f>IF(K93="","",IFERROR(VLOOKUP(J93,Fiat!$B$1:$C$20,2,FALSE)*K93,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5121,11 +5024,11 @@
         <f t="array" ref="J94">IFERROR(_FV(C94,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K94" s="31" t="str" cm="1">
+      <c r="K94" s="25" t="str" cm="1">
         <f t="array" ref="K94">IFERROR(_FV(C94,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L94" s="31" t="str">
+      <c r="L94" s="25" t="str">
         <f>IF(K94="","",IFERROR(VLOOKUP(J94,Fiat!$B$1:$C$20,2,FALSE)*K94,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5158,11 +5061,11 @@
         <f t="array" ref="J95">IFERROR(_FV(C95,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K95" s="31" t="str" cm="1">
+      <c r="K95" s="25" t="str" cm="1">
         <f t="array" ref="K95">IFERROR(_FV(C95,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L95" s="31" t="str">
+      <c r="L95" s="25" t="str">
         <f>IF(K95="","",IFERROR(VLOOKUP(J95,Fiat!$B$1:$C$20,2,FALSE)*K95,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5195,11 +5098,11 @@
         <f t="array" ref="J96">IFERROR(_FV(C96,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K96" s="31" t="str" cm="1">
+      <c r="K96" s="25" t="str" cm="1">
         <f t="array" ref="K96">IFERROR(_FV(C96,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L96" s="31" t="str">
+      <c r="L96" s="25" t="str">
         <f>IF(K96="","",IFERROR(VLOOKUP(J96,Fiat!$B$1:$C$20,2,FALSE)*K96,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5232,11 +5135,11 @@
         <f t="array" ref="J97">IFERROR(_FV(C97,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K97" s="31" t="str" cm="1">
+      <c r="K97" s="25" t="str" cm="1">
         <f t="array" ref="K97">IFERROR(_FV(C97,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L97" s="31" t="str">
+      <c r="L97" s="25" t="str">
         <f>IF(K97="","",IFERROR(VLOOKUP(J97,Fiat!$B$1:$C$20,2,FALSE)*K97,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5254,7 +5157,7 @@
     </row>
     <row r="98" spans="1:17">
       <c r="A98" s="9" t="str">
-        <f t="shared" ref="A98:A129" si="3">IF(B98="","",ROW()-1)</f>
+        <f t="shared" ref="A98:A121" si="3">IF(B98="","",ROW()-1)</f>
         <v/>
       </c>
       <c r="B98" s="15"/>
@@ -5269,11 +5172,11 @@
         <f t="array" ref="J98">IFERROR(_FV(C98,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K98" s="31" t="str" cm="1">
+      <c r="K98" s="25" t="str" cm="1">
         <f t="array" ref="K98">IFERROR(_FV(C98,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L98" s="31" t="str">
+      <c r="L98" s="25" t="str">
         <f>IF(K98="","",IFERROR(VLOOKUP(J98,Fiat!$B$1:$C$20,2,FALSE)*K98,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5306,11 +5209,11 @@
         <f t="array" ref="J99">IFERROR(_FV(C99,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K99" s="31" t="str" cm="1">
+      <c r="K99" s="25" t="str" cm="1">
         <f t="array" ref="K99">IFERROR(_FV(C99,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L99" s="31" t="str">
+      <c r="L99" s="25" t="str">
         <f>IF(K99="","",IFERROR(VLOOKUP(J99,Fiat!$B$1:$C$20,2,FALSE)*K99,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5343,11 +5246,11 @@
         <f t="array" ref="J100">IFERROR(_FV(C100,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K100" s="31" t="str" cm="1">
+      <c r="K100" s="25" t="str" cm="1">
         <f t="array" ref="K100">IFERROR(_FV(C100,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L100" s="31" t="str">
+      <c r="L100" s="25" t="str">
         <f>IF(K100="","",IFERROR(VLOOKUP(J100,Fiat!$B$1:$C$20,2,FALSE)*K100,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5380,11 +5283,11 @@
         <f t="array" ref="J101">IFERROR(_FV(C101,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K101" s="31" t="str" cm="1">
+      <c r="K101" s="25" t="str" cm="1">
         <f t="array" ref="K101">IFERROR(_FV(C101,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L101" s="31" t="str">
+      <c r="L101" s="25" t="str">
         <f>IF(K101="","",IFERROR(VLOOKUP(J101,Fiat!$B$1:$C$20,2,FALSE)*K101,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5417,11 +5320,11 @@
         <f t="array" ref="J102">IFERROR(_FV(C102,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K102" s="31" t="str" cm="1">
+      <c r="K102" s="25" t="str" cm="1">
         <f t="array" ref="K102">IFERROR(_FV(C102,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L102" s="31" t="str">
+      <c r="L102" s="25" t="str">
         <f>IF(K102="","",IFERROR(VLOOKUP(J102,Fiat!$B$1:$C$20,2,FALSE)*K102,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5454,11 +5357,11 @@
         <f t="array" ref="J103">IFERROR(_FV(C103,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K103" s="31" t="str" cm="1">
+      <c r="K103" s="25" t="str" cm="1">
         <f t="array" ref="K103">IFERROR(_FV(C103,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L103" s="31" t="str">
+      <c r="L103" s="25" t="str">
         <f>IF(K103="","",IFERROR(VLOOKUP(J103,Fiat!$B$1:$C$20,2,FALSE)*K103,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5491,11 +5394,11 @@
         <f t="array" ref="J104">IFERROR(_FV(C104,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K104" s="31" t="str" cm="1">
+      <c r="K104" s="25" t="str" cm="1">
         <f t="array" ref="K104">IFERROR(_FV(C104,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L104" s="31" t="str">
+      <c r="L104" s="25" t="str">
         <f>IF(K104="","",IFERROR(VLOOKUP(J104,Fiat!$B$1:$C$20,2,FALSE)*K104,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5528,11 +5431,11 @@
         <f t="array" ref="J105">IFERROR(_FV(C105,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K105" s="31" t="str" cm="1">
+      <c r="K105" s="25" t="str" cm="1">
         <f t="array" ref="K105">IFERROR(_FV(C105,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L105" s="31" t="str">
+      <c r="L105" s="25" t="str">
         <f>IF(K105="","",IFERROR(VLOOKUP(J105,Fiat!$B$1:$C$20,2,FALSE)*K105,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5565,11 +5468,11 @@
         <f t="array" ref="J106">IFERROR(_FV(C106,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K106" s="31" t="str" cm="1">
+      <c r="K106" s="25" t="str" cm="1">
         <f t="array" ref="K106">IFERROR(_FV(C106,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L106" s="31" t="str">
+      <c r="L106" s="25" t="str">
         <f>IF(K106="","",IFERROR(VLOOKUP(J106,Fiat!$B$1:$C$20,2,FALSE)*K106,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5602,11 +5505,11 @@
         <f t="array" ref="J107">IFERROR(_FV(C107,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K107" s="31" t="str" cm="1">
+      <c r="K107" s="25" t="str" cm="1">
         <f t="array" ref="K107">IFERROR(_FV(C107,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L107" s="31" t="str">
+      <c r="L107" s="25" t="str">
         <f>IF(K107="","",IFERROR(VLOOKUP(J107,Fiat!$B$1:$C$20,2,FALSE)*K107,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5639,11 +5542,11 @@
         <f t="array" ref="J108">IFERROR(_FV(C108,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K108" s="31" t="str" cm="1">
+      <c r="K108" s="25" t="str" cm="1">
         <f t="array" ref="K108">IFERROR(_FV(C108,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L108" s="31" t="str">
+      <c r="L108" s="25" t="str">
         <f>IF(K108="","",IFERROR(VLOOKUP(J108,Fiat!$B$1:$C$20,2,FALSE)*K108,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5676,11 +5579,11 @@
         <f t="array" ref="J109">IFERROR(_FV(C109,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K109" s="31" t="str" cm="1">
+      <c r="K109" s="25" t="str" cm="1">
         <f t="array" ref="K109">IFERROR(_FV(C109,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L109" s="31" t="str">
+      <c r="L109" s="25" t="str">
         <f>IF(K109="","",IFERROR(VLOOKUP(J109,Fiat!$B$1:$C$20,2,FALSE)*K109,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5713,11 +5616,11 @@
         <f t="array" ref="J110">IFERROR(_FV(C110,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K110" s="31" t="str" cm="1">
+      <c r="K110" s="25" t="str" cm="1">
         <f t="array" ref="K110">IFERROR(_FV(C110,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L110" s="31" t="str">
+      <c r="L110" s="25" t="str">
         <f>IF(K110="","",IFERROR(VLOOKUP(J110,Fiat!$B$1:$C$20,2,FALSE)*K110,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5750,11 +5653,11 @@
         <f t="array" ref="J111">IFERROR(_FV(C111,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K111" s="31" t="str" cm="1">
+      <c r="K111" s="25" t="str" cm="1">
         <f t="array" ref="K111">IFERROR(_FV(C111,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L111" s="31" t="str">
+      <c r="L111" s="25" t="str">
         <f>IF(K111="","",IFERROR(VLOOKUP(J111,Fiat!$B$1:$C$20,2,FALSE)*K111,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5787,11 +5690,11 @@
         <f t="array" ref="J112">IFERROR(_FV(C112,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K112" s="31" t="str" cm="1">
+      <c r="K112" s="25" t="str" cm="1">
         <f t="array" ref="K112">IFERROR(_FV(C112,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L112" s="31" t="str">
+      <c r="L112" s="25" t="str">
         <f>IF(K112="","",IFERROR(VLOOKUP(J112,Fiat!$B$1:$C$20,2,FALSE)*K112,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5824,11 +5727,11 @@
         <f t="array" ref="J113">IFERROR(_FV(C113,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K113" s="31" t="str" cm="1">
+      <c r="K113" s="25" t="str" cm="1">
         <f t="array" ref="K113">IFERROR(_FV(C113,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L113" s="31" t="str">
+      <c r="L113" s="25" t="str">
         <f>IF(K113="","",IFERROR(VLOOKUP(J113,Fiat!$B$1:$C$20,2,FALSE)*K113,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5861,11 +5764,11 @@
         <f t="array" ref="J114">IFERROR(_FV(C114,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K114" s="31" t="str" cm="1">
+      <c r="K114" s="25" t="str" cm="1">
         <f t="array" ref="K114">IFERROR(_FV(C114,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L114" s="31" t="str">
+      <c r="L114" s="25" t="str">
         <f>IF(K114="","",IFERROR(VLOOKUP(J114,Fiat!$B$1:$C$20,2,FALSE)*K114,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5898,11 +5801,11 @@
         <f t="array" ref="J115">IFERROR(_FV(C115,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K115" s="31" t="str" cm="1">
+      <c r="K115" s="25" t="str" cm="1">
         <f t="array" ref="K115">IFERROR(_FV(C115,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L115" s="31" t="str">
+      <c r="L115" s="25" t="str">
         <f>IF(K115="","",IFERROR(VLOOKUP(J115,Fiat!$B$1:$C$20,2,FALSE)*K115,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5935,11 +5838,11 @@
         <f t="array" ref="J116">IFERROR(_FV(C116,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K116" s="31" t="str" cm="1">
+      <c r="K116" s="25" t="str" cm="1">
         <f t="array" ref="K116">IFERROR(_FV(C116,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L116" s="31" t="str">
+      <c r="L116" s="25" t="str">
         <f>IF(K116="","",IFERROR(VLOOKUP(J116,Fiat!$B$1:$C$20,2,FALSE)*K116,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -5972,11 +5875,11 @@
         <f t="array" ref="J117">IFERROR(_FV(C117,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K117" s="31" t="str" cm="1">
+      <c r="K117" s="25" t="str" cm="1">
         <f t="array" ref="K117">IFERROR(_FV(C117,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L117" s="31" t="str">
+      <c r="L117" s="25" t="str">
         <f>IF(K117="","",IFERROR(VLOOKUP(J117,Fiat!$B$1:$C$20,2,FALSE)*K117,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -6009,11 +5912,11 @@
         <f t="array" ref="J118">IFERROR(_FV(C118,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K118" s="31" t="str" cm="1">
+      <c r="K118" s="25" t="str" cm="1">
         <f t="array" ref="K118">IFERROR(_FV(C118,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L118" s="31" t="str">
+      <c r="L118" s="25" t="str">
         <f>IF(K118="","",IFERROR(VLOOKUP(J118,Fiat!$B$1:$C$20,2,FALSE)*K118,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -6046,11 +5949,11 @@
         <f t="array" ref="J119">IFERROR(_FV(C119,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K119" s="31" t="str" cm="1">
+      <c r="K119" s="25" t="str" cm="1">
         <f t="array" ref="K119">IFERROR(_FV(C119,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L119" s="31" t="str">
+      <c r="L119" s="25" t="str">
         <f>IF(K119="","",IFERROR(VLOOKUP(J119,Fiat!$B$1:$C$20,2,FALSE)*K119,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -6083,11 +5986,11 @@
         <f t="array" ref="J120">IFERROR(_FV(C120,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K120" s="31" t="str" cm="1">
+      <c r="K120" s="25" t="str" cm="1">
         <f t="array" ref="K120">IFERROR(_FV(C120,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L120" s="31" t="str">
+      <c r="L120" s="25" t="str">
         <f>IF(K120="","",IFERROR(VLOOKUP(J120,Fiat!$B$1:$C$20,2,FALSE)*K120,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -6120,11 +6023,11 @@
         <f t="array" ref="J121">IFERROR(_FV(C121,"Currency"),"")</f>
         <v/>
       </c>
-      <c r="K121" s="31" t="str" cm="1">
+      <c r="K121" s="25" t="str" cm="1">
         <f t="array" ref="K121">IFERROR(_FV(C121,"Market cap",TRUE)/1000000,"")</f>
         <v/>
       </c>
-      <c r="L121" s="31" t="str">
+      <c r="L121" s="25" t="str">
         <f>IF(K121="","",IFERROR(VLOOKUP(J121,Fiat!$B$1:$C$20,2,FALSE)*K121,"Valuta ontbreekt op Fiat"))</f>
         <v/>
       </c>
@@ -6189,7 +6092,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="B1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C1">
         <v>1</v>
@@ -6200,7 +6103,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C2" s="7" cm="1">
         <f t="array" aca="1" ref="C2" ca="1">_FV(A2,"Price")</f>
@@ -6212,7 +6115,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C3" s="7" cm="1">
         <f t="array" aca="1" ref="C3" ca="1">_FV(A3,"Price")</f>
@@ -6224,7 +6127,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C4" s="7" cm="1">
         <f t="array" aca="1" ref="C4" ca="1">_FV(A4,"Price")</f>
@@ -6236,7 +6139,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C5" s="7" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(A5,"Price")</f>
@@ -6293,10 +6196,10 @@
         <v>32</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>33</v>
+        <v>112</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="89.25">
@@ -6304,16 +6207,16 @@
         <v>12</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>32</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="76.5">
@@ -6321,16 +6224,16 @@
         <v>13</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>32</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="51">
@@ -6338,16 +6241,16 @@
         <v>14</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="51">
@@ -6355,16 +6258,16 @@
         <v>15</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>42</v>
-      </c>
       <c r="E6" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="38.25">
@@ -6372,16 +6275,16 @@
         <v>16</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>32</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="63.75">
@@ -6389,33 +6292,33 @@
         <v>17</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>32</v>
       </c>
       <c r="D8" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="102">
       <c r="A9" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>99</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>100</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>32</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>101</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="25.5">
@@ -6423,16 +6326,16 @@
         <v>18</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>49</v>
-      </c>
       <c r="E10" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="25.5">
@@ -6440,16 +6343,16 @@
         <v>19</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>51</v>
-      </c>
       <c r="E11" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="25.5">
@@ -6457,27 +6360,27 @@
         <v>20</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="48" customHeight="1"/>
     <row r="14" spans="1:5" ht="48" customHeight="1">
-      <c r="A14" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="B14" s="34"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
+      <c r="A14" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" s="31"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6503,28 +6406,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24">
-      <c r="A1" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
+      <c r="A1" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
+      <c r="A2" s="35" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="20"/>
@@ -6538,43 +6441,43 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B4" s="21"/>
       <c r="C4" s="21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D4" s="21"/>
       <c r="E4" s="21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F4" s="21"/>
       <c r="G4" s="21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:8" ht="26.25">
-      <c r="A5" s="26">
+      <c r="A5" s="36">
         <f>COUNTA(Kandidaten!$B$2:$B$121)</f>
         <v>0</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26" cm="1">
+      <c r="B5" s="36"/>
+      <c r="C5" s="36" cm="1">
         <f t="array" ref="C5">IFERROR(ROWS(_xlfn.UNIQUE(_xlfn._xlws.FILTER(Kandidaten!$E$2:$E$121,Kandidaten!$B$2:$B$121&lt;&gt;""))),0)</f>
         <v>0</v>
       </c>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26" cm="1">
+      <c r="D5" s="36"/>
+      <c r="E5" s="36" cm="1">
         <f t="array" ref="E5">IFERROR(ROWS(_xlfn.UNIQUE(_xlfn._xlws.FILTER(Kandidaten!$G$2:$G$121,Kandidaten!$B$2:$B$121&lt;&gt;""))),0)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="26"/>
-      <c r="G5" s="27">
+      <c r="F5" s="36"/>
+      <c r="G5" s="37">
         <f>IF(A5=0,0,COUNTIFS(Kandidaten!$B$2:$B$121,"&lt;&gt;",Kandidaten!$D$2:$D$121,"&lt;&gt;",Kandidaten!$E$2:$E$121,"&lt;&gt;",Kandidaten!$F$2:$F$121,"&lt;&gt;",Kandidaten!$G$2:$G$121,"&lt;&gt;",Kandidaten!$O$2:$O$121,"&lt;&gt;",Kandidaten!$P$2:$P$121,"&lt;&gt;",Kandidaten!$Q$2:$Q$121,"&lt;&gt;")/A5)</f>
         <v>0</v>
       </c>
-      <c r="H5" s="27"/>
+      <c r="H5" s="37"/>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="20"/>
@@ -6587,56 +6490,56 @@
       <c r="H6" s="20"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="28" t="s">
-        <v>74</v>
-      </c>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
+      <c r="A7" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="B7" s="32"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B8" s="21"/>
       <c r="C8" s="21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D8" s="21"/>
       <c r="E8" s="21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="21" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" ht="21">
-      <c r="A9" s="29">
+      <c r="A9" s="33">
         <f>COUNTIFS(Kandidaten!$B$2:$B$121,"&lt;&gt;",Kandidaten!$O$2:$O$121,"")</f>
         <v>0</v>
       </c>
-      <c r="B9" s="29"/>
-      <c r="C9" s="29">
+      <c r="B9" s="33"/>
+      <c r="C9" s="33">
         <f>COUNTIFS(Kandidaten!$B$2:$B$121,"&lt;&gt;",Kandidaten!$P$2:$P$121,"")</f>
         <v>0</v>
       </c>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29">
+      <c r="D9" s="33"/>
+      <c r="E9" s="33">
         <f>COUNTIFS(Kandidaten!$B$2:$B$121,"&lt;&gt;",Kandidaten!$Q$2:$Q$121,"")</f>
         <v>0</v>
       </c>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29">
+      <c r="F9" s="33"/>
+      <c r="G9" s="33">
         <f>COUNTIFS(Kandidaten!$B$2:$B$121,"&lt;&gt;",Kandidaten!$D$2:$D$121,"")</f>
         <v>0</v>
       </c>
-      <c r="H9" s="29"/>
+      <c r="H9" s="33"/>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="20"/>
@@ -6650,24 +6553,24 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" s="22" t="s">
         <v>79</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>80</v>
       </c>
       <c r="C11" s="20"/>
       <c r="D11" s="22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F11" s="20"/>
       <c r="G11" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H11" s="22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -6980,17 +6883,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G9:H9"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="G5:H5"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G9:H9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>